<commit_message>
July1 2024 changes 2
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFD8B96-7234-4DE4-84CE-45F817672EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FA17C0-8441-424F-A3AA-65E0EBE4B4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -86,9 +86,6 @@
     <t>JobType</t>
   </si>
   <si>
-    <t>IndustryGroup</t>
-  </si>
-  <si>
     <t>Sector</t>
   </si>
   <si>
@@ -299,14 +296,17 @@
     <t>Advisory (CF)</t>
   </si>
   <si>
-    <t>Business Services</t>
+    <t>CSDN-0000007327</t>
+  </si>
+  <si>
+    <t>IndustryGroup/HLSector</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,6 +318,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -637,13 +643,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -651,7 +657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -667,12 +673,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -680,7 +686,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -696,17 +702,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -719,17 +725,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -743,15 +749,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -762,1323 +768,1324 @@
         <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AD1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" t="s">
-        <v>42</v>
-      </c>
       <c r="F2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" t="s">
         <v>43</v>
       </c>
-      <c r="G2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" t="s">
         <v>44</v>
       </c>
-      <c r="I2" t="s">
-        <v>43</v>
-      </c>
-      <c r="J2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>45</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>46</v>
       </c>
-      <c r="M2" t="s">
-        <v>47</v>
-      </c>
       <c r="N2" t="s">
         <v>0</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R2" t="s">
+        <v>48</v>
+      </c>
+      <c r="S2" t="s">
+        <v>48</v>
+      </c>
+      <c r="T2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S2" t="s">
-        <v>49</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" t="s">
         <v>50</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>51</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>52</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>53</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>54</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>55</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="s">
         <v>56</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>57</v>
       </c>
       <c r="AE2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" t="s">
         <v>41</v>
       </c>
-      <c r="B3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" t="s">
-        <v>42</v>
-      </c>
       <c r="F3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" t="s">
         <v>43</v>
       </c>
-      <c r="G3" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J3" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" t="s">
         <v>44</v>
       </c>
-      <c r="I3" t="s">
-        <v>43</v>
-      </c>
-      <c r="J3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>45</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>46</v>
       </c>
-      <c r="M3" t="s">
-        <v>47</v>
-      </c>
       <c r="N3" t="s">
         <v>0</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R3" t="s">
+        <v>48</v>
+      </c>
+      <c r="S3" t="s">
+        <v>48</v>
+      </c>
+      <c r="T3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S3" t="s">
-        <v>49</v>
-      </c>
-      <c r="T3" s="3" t="s">
+      <c r="U3" t="s">
         <v>50</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>51</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>52</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>53</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Y3" t="s">
         <v>54</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>55</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="s">
         <v>56</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>57</v>
       </c>
       <c r="AE3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
       <c r="F4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" t="s">
         <v>43</v>
       </c>
-      <c r="G4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" t="s">
         <v>44</v>
       </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
-        <v>43</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>45</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>46</v>
       </c>
-      <c r="M4" t="s">
-        <v>47</v>
-      </c>
       <c r="N4" t="s">
         <v>0</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R4" t="s">
+        <v>48</v>
+      </c>
+      <c r="S4" t="s">
+        <v>48</v>
+      </c>
+      <c r="T4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S4" t="s">
-        <v>49</v>
-      </c>
-      <c r="T4" s="3" t="s">
+      <c r="U4" t="s">
         <v>50</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>51</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" t="s">
         <v>52</v>
       </c>
-      <c r="W4" t="s">
+      <c r="X4" t="s">
         <v>53</v>
       </c>
-      <c r="X4" t="s">
+      <c r="Y4" t="s">
         <v>54</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>55</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="s">
         <v>56</v>
-      </c>
-      <c r="AA4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>57</v>
       </c>
       <c r="AE4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" t="s">
         <v>41</v>
       </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" t="s">
-        <v>42</v>
-      </c>
       <c r="F5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" t="s">
         <v>43</v>
       </c>
-      <c r="G5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K5" t="s">
         <v>44</v>
       </c>
-      <c r="I5" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" t="s">
-        <v>43</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>45</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>46</v>
       </c>
-      <c r="M5" t="s">
-        <v>47</v>
-      </c>
       <c r="N5" t="s">
         <v>0</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R5" t="s">
+        <v>48</v>
+      </c>
+      <c r="S5" t="s">
+        <v>48</v>
+      </c>
+      <c r="T5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S5" t="s">
-        <v>49</v>
-      </c>
-      <c r="T5" s="3" t="s">
+      <c r="U5" t="s">
         <v>50</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>51</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>52</v>
       </c>
-      <c r="W5" t="s">
+      <c r="X5" t="s">
         <v>53</v>
       </c>
-      <c r="X5" t="s">
+      <c r="Y5" t="s">
         <v>54</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>55</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="s">
         <v>56</v>
-      </c>
-      <c r="AA5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>57</v>
       </c>
       <c r="AE5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" t="s">
-        <v>42</v>
-      </c>
       <c r="F6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
         <v>43</v>
       </c>
-      <c r="G6" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" t="s">
         <v>44</v>
       </c>
-      <c r="I6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J6" t="s">
-        <v>43</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>45</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>46</v>
       </c>
-      <c r="M6" t="s">
-        <v>47</v>
-      </c>
       <c r="N6" t="s">
         <v>0</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R6" t="s">
+        <v>48</v>
+      </c>
+      <c r="S6" t="s">
+        <v>48</v>
+      </c>
+      <c r="T6" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S6" t="s">
-        <v>49</v>
-      </c>
-      <c r="T6" s="3" t="s">
+      <c r="U6" t="s">
         <v>50</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>51</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>52</v>
       </c>
-      <c r="W6" t="s">
+      <c r="X6" t="s">
         <v>53</v>
       </c>
-      <c r="X6" t="s">
+      <c r="Y6" t="s">
         <v>54</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>55</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="s">
         <v>56</v>
-      </c>
-      <c r="AA6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>57</v>
       </c>
       <c r="AE6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E7" t="s">
         <v>41</v>
       </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" t="s">
-        <v>85</v>
-      </c>
-      <c r="E7" t="s">
-        <v>42</v>
-      </c>
       <c r="F7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K7" t="s">
         <v>44</v>
       </c>
-      <c r="I7" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>45</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>46</v>
       </c>
-      <c r="M7" t="s">
-        <v>47</v>
-      </c>
       <c r="N7" t="s">
         <v>0</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R7" t="s">
+        <v>48</v>
+      </c>
+      <c r="S7" t="s">
+        <v>48</v>
+      </c>
+      <c r="T7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S7" t="s">
-        <v>49</v>
-      </c>
-      <c r="T7" s="3" t="s">
+      <c r="U7" t="s">
         <v>50</v>
       </c>
-      <c r="U7" t="s">
+      <c r="V7" t="s">
         <v>51</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>52</v>
       </c>
-      <c r="W7" t="s">
+      <c r="X7" t="s">
         <v>53</v>
       </c>
-      <c r="X7" t="s">
+      <c r="Y7" t="s">
         <v>54</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Z7" t="s">
         <v>55</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="s">
         <v>56</v>
-      </c>
-      <c r="AA7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="s">
-        <v>57</v>
       </c>
       <c r="AE7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D8" t="s">
-        <v>85</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
       <c r="F8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H8" t="s">
         <v>43</v>
       </c>
-      <c r="G8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
+        <v>42</v>
+      </c>
+      <c r="J8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" t="s">
         <v>44</v>
       </c>
-      <c r="I8" t="s">
-        <v>43</v>
-      </c>
-      <c r="J8" t="s">
-        <v>43</v>
-      </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>45</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>46</v>
       </c>
-      <c r="M8" t="s">
-        <v>47</v>
-      </c>
       <c r="N8" t="s">
         <v>0</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R8" t="s">
+        <v>48</v>
+      </c>
+      <c r="S8" t="s">
+        <v>48</v>
+      </c>
+      <c r="T8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S8" t="s">
-        <v>49</v>
-      </c>
-      <c r="T8" s="3" t="s">
+      <c r="U8" t="s">
         <v>50</v>
       </c>
-      <c r="U8" t="s">
+      <c r="V8" t="s">
         <v>51</v>
       </c>
-      <c r="V8" t="s">
+      <c r="W8" t="s">
         <v>52</v>
       </c>
-      <c r="W8" t="s">
+      <c r="X8" t="s">
         <v>53</v>
       </c>
-      <c r="X8" t="s">
+      <c r="Y8" t="s">
         <v>54</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Z8" t="s">
         <v>55</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="s">
         <v>56</v>
-      </c>
-      <c r="AA8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC8" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>57</v>
       </c>
       <c r="AE8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" t="s">
         <v>41</v>
       </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D9" t="s">
-        <v>85</v>
-      </c>
-      <c r="E9" t="s">
-        <v>42</v>
-      </c>
       <c r="F9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H9" t="s">
         <v>43</v>
       </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" t="s">
         <v>44</v>
       </c>
-      <c r="I9" t="s">
-        <v>43</v>
-      </c>
-      <c r="J9" t="s">
-        <v>43</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>45</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>46</v>
       </c>
-      <c r="M9" t="s">
-        <v>47</v>
-      </c>
       <c r="N9" t="s">
         <v>0</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R9" t="s">
+        <v>48</v>
+      </c>
+      <c r="S9" t="s">
+        <v>48</v>
+      </c>
+      <c r="T9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S9" t="s">
-        <v>49</v>
-      </c>
-      <c r="T9" s="3" t="s">
+      <c r="U9" t="s">
         <v>50</v>
       </c>
-      <c r="U9" t="s">
+      <c r="V9" t="s">
         <v>51</v>
       </c>
-      <c r="V9" t="s">
+      <c r="W9" t="s">
         <v>52</v>
       </c>
-      <c r="W9" t="s">
+      <c r="X9" t="s">
         <v>53</v>
       </c>
-      <c r="X9" t="s">
+      <c r="Y9" t="s">
         <v>54</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Z9" t="s">
         <v>55</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="s">
         <v>56</v>
-      </c>
-      <c r="AA9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC9" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>57</v>
       </c>
       <c r="AE9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" t="s">
         <v>41</v>
       </c>
-      <c r="B10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D10" t="s">
-        <v>85</v>
-      </c>
-      <c r="E10" t="s">
-        <v>42</v>
-      </c>
       <c r="F10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" t="s">
+        <v>42</v>
+      </c>
+      <c r="H10" t="s">
         <v>43</v>
       </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K10" t="s">
         <v>44</v>
       </c>
-      <c r="I10" t="s">
-        <v>43</v>
-      </c>
-      <c r="J10" t="s">
-        <v>43</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>45</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>46</v>
       </c>
-      <c r="M10" t="s">
-        <v>47</v>
-      </c>
       <c r="N10" t="s">
         <v>0</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R10" t="s">
+        <v>48</v>
+      </c>
+      <c r="S10" t="s">
+        <v>48</v>
+      </c>
+      <c r="T10" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S10" t="s">
-        <v>49</v>
-      </c>
-      <c r="T10" s="3" t="s">
+      <c r="U10" t="s">
         <v>50</v>
       </c>
-      <c r="U10" t="s">
+      <c r="V10" t="s">
         <v>51</v>
       </c>
-      <c r="V10" t="s">
+      <c r="W10" t="s">
         <v>52</v>
       </c>
-      <c r="W10" t="s">
+      <c r="X10" t="s">
         <v>53</v>
       </c>
-      <c r="X10" t="s">
+      <c r="Y10" t="s">
         <v>54</v>
       </c>
-      <c r="Y10" t="s">
+      <c r="Z10" t="s">
         <v>55</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="AA10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="s">
         <v>56</v>
-      </c>
-      <c r="AA10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC10" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>57</v>
       </c>
       <c r="AE10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D11" t="s">
-        <v>85</v>
-      </c>
-      <c r="E11" t="s">
-        <v>42</v>
-      </c>
       <c r="F11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H11" t="s">
         <v>43</v>
       </c>
-      <c r="G11" t="s">
-        <v>43</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" t="s">
+        <v>42</v>
+      </c>
+      <c r="K11" t="s">
         <v>44</v>
       </c>
-      <c r="I11" t="s">
-        <v>43</v>
-      </c>
-      <c r="J11" t="s">
-        <v>43</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>45</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>46</v>
       </c>
-      <c r="M11" t="s">
-        <v>47</v>
-      </c>
       <c r="N11" t="s">
         <v>0</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R11" t="s">
+        <v>48</v>
+      </c>
+      <c r="S11" t="s">
+        <v>48</v>
+      </c>
+      <c r="T11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S11" t="s">
-        <v>49</v>
-      </c>
-      <c r="T11" s="3" t="s">
+      <c r="U11" t="s">
         <v>50</v>
       </c>
-      <c r="U11" t="s">
+      <c r="V11" t="s">
         <v>51</v>
       </c>
-      <c r="V11" t="s">
+      <c r="W11" t="s">
         <v>52</v>
       </c>
-      <c r="W11" t="s">
+      <c r="X11" t="s">
         <v>53</v>
       </c>
-      <c r="X11" t="s">
+      <c r="Y11" t="s">
         <v>54</v>
       </c>
-      <c r="Y11" t="s">
+      <c r="Z11" t="s">
         <v>55</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="AA11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="s">
         <v>56</v>
-      </c>
-      <c r="AA11" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB11" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>57</v>
       </c>
       <c r="AE11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" t="s">
         <v>41</v>
       </c>
-      <c r="B12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" t="s">
-        <v>42</v>
-      </c>
       <c r="F12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H12" t="s">
         <v>43</v>
       </c>
-      <c r="G12" t="s">
-        <v>43</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
+        <v>42</v>
+      </c>
+      <c r="J12" t="s">
+        <v>42</v>
+      </c>
+      <c r="K12" t="s">
         <v>44</v>
       </c>
-      <c r="I12" t="s">
-        <v>43</v>
-      </c>
-      <c r="J12" t="s">
-        <v>43</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>45</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>46</v>
       </c>
-      <c r="M12" t="s">
-        <v>47</v>
-      </c>
       <c r="N12" t="s">
         <v>0</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R12" t="s">
+        <v>48</v>
+      </c>
+      <c r="S12" t="s">
+        <v>48</v>
+      </c>
+      <c r="T12" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S12" t="s">
-        <v>49</v>
-      </c>
-      <c r="T12" s="3" t="s">
+      <c r="U12" t="s">
         <v>50</v>
       </c>
-      <c r="U12" t="s">
+      <c r="V12" t="s">
         <v>51</v>
       </c>
-      <c r="V12" t="s">
+      <c r="W12" t="s">
         <v>52</v>
       </c>
-      <c r="W12" t="s">
+      <c r="X12" t="s">
         <v>53</v>
       </c>
-      <c r="X12" t="s">
+      <c r="Y12" t="s">
         <v>54</v>
       </c>
-      <c r="Y12" t="s">
+      <c r="Z12" t="s">
         <v>55</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="AA12" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB12" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="s">
         <v>56</v>
-      </c>
-      <c r="AA12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC12" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD12" t="s">
-        <v>57</v>
       </c>
       <c r="AE12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="D13" t="s">
-        <v>85</v>
-      </c>
-      <c r="E13" t="s">
-        <v>42</v>
-      </c>
       <c r="F13" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" t="s">
         <v>43</v>
       </c>
-      <c r="G13" t="s">
-        <v>43</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" t="s">
         <v>44</v>
       </c>
-      <c r="I13" t="s">
-        <v>43</v>
-      </c>
-      <c r="J13" t="s">
-        <v>43</v>
-      </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>45</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>46</v>
       </c>
-      <c r="M13" t="s">
-        <v>47</v>
-      </c>
       <c r="N13" t="s">
         <v>0</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R13" t="s">
+        <v>48</v>
+      </c>
+      <c r="S13" t="s">
+        <v>48</v>
+      </c>
+      <c r="T13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S13" t="s">
-        <v>49</v>
-      </c>
-      <c r="T13" s="3" t="s">
+      <c r="U13" t="s">
         <v>50</v>
       </c>
-      <c r="U13" t="s">
+      <c r="V13" t="s">
         <v>51</v>
       </c>
-      <c r="V13" t="s">
+      <c r="W13" t="s">
         <v>52</v>
       </c>
-      <c r="W13" t="s">
+      <c r="X13" t="s">
         <v>53</v>
       </c>
-      <c r="X13" t="s">
+      <c r="Y13" t="s">
         <v>54</v>
       </c>
-      <c r="Y13" t="s">
+      <c r="Z13" t="s">
         <v>55</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="AA13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="s">
         <v>56</v>
-      </c>
-      <c r="AA13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC13" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD13" t="s">
-        <v>57</v>
       </c>
       <c r="AE13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14" t="s">
-        <v>85</v>
-      </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
       <c r="F14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" t="s">
         <v>43</v>
       </c>
-      <c r="G14" t="s">
-        <v>43</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
+        <v>42</v>
+      </c>
+      <c r="J14" t="s">
+        <v>42</v>
+      </c>
+      <c r="K14" t="s">
         <v>44</v>
       </c>
-      <c r="I14" t="s">
-        <v>43</v>
-      </c>
-      <c r="J14" t="s">
-        <v>43</v>
-      </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>45</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>46</v>
       </c>
-      <c r="M14" t="s">
-        <v>47</v>
-      </c>
       <c r="N14" t="s">
         <v>0</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R14" t="s">
+        <v>48</v>
+      </c>
+      <c r="S14" t="s">
+        <v>48</v>
+      </c>
+      <c r="T14" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S14" t="s">
-        <v>49</v>
-      </c>
-      <c r="T14" s="3" t="s">
+      <c r="U14" t="s">
         <v>50</v>
       </c>
-      <c r="U14" t="s">
+      <c r="V14" t="s">
         <v>51</v>
       </c>
-      <c r="V14" t="s">
+      <c r="W14" t="s">
         <v>52</v>
       </c>
-      <c r="W14" t="s">
+      <c r="X14" t="s">
         <v>53</v>
       </c>
-      <c r="X14" t="s">
+      <c r="Y14" t="s">
         <v>54</v>
       </c>
-      <c r="Y14" t="s">
+      <c r="Z14" t="s">
         <v>55</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="AA14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="s">
         <v>56</v>
-      </c>
-      <c r="AA14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC14" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD14" t="s">
-        <v>57</v>
       </c>
       <c r="AE14">
         <v>13</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2087,68 +2094,68 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>65</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>66</v>
-      </c>
-      <c r="D2" t="s">
-        <v>67</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2159,158 +2166,158 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" t="s">
         <v>70</v>
-      </c>
-      <c r="B3" t="s">
-        <v>71</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>84</v>
       </c>
       <c r="C14">
         <v>13</v>

</xml_diff>

<commit_message>
CDSN changes data and function changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FA17C0-8441-424F-A3AA-65E0EBE4B4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616FD5A7-B7FB-4C0C-9B8C-64ED8781F918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -296,10 +296,10 @@
     <t>Advisory (CF)</t>
   </si>
   <si>
-    <t>CSDN-0000007327</t>
-  </si>
-  <si>
     <t>IndustryGroup/HLSector</t>
+  </si>
+  <si>
+    <t>CSDN-0000002536</t>
   </si>
 </sst>
 </file>
@@ -643,13 +643,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -657,7 +657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -673,12 +673,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -686,7 +686,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -702,17 +702,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -725,17 +725,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -749,15 +749,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -768,7 +768,7 @@
         <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>14</v>
@@ -849,7 +849,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -860,7 +860,7 @@
         <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" t="s">
         <v>41</v>
@@ -944,7 +944,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -955,7 +955,7 @@
         <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
         <v>41</v>
@@ -1039,7 +1039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>71</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E4" t="s">
         <v>41</v>
@@ -1134,7 +1134,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>73</v>
       </c>
       <c r="D5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E5" t="s">
         <v>41</v>
@@ -1229,7 +1229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E6" t="s">
         <v>41</v>
@@ -1324,7 +1324,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E7" t="s">
         <v>41</v>
@@ -1419,7 +1419,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>76</v>
       </c>
       <c r="D8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E8" t="s">
         <v>41</v>
@@ -1514,7 +1514,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>77</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E9" t="s">
         <v>41</v>
@@ -1609,7 +1609,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>78</v>
       </c>
       <c r="D10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E10" t="s">
         <v>41</v>
@@ -1704,7 +1704,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>79</v>
       </c>
       <c r="D11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E11" t="s">
         <v>41</v>
@@ -1799,7 +1799,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>80</v>
       </c>
       <c r="D12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E12" t="s">
         <v>41</v>
@@ -1894,7 +1894,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>81</v>
       </c>
       <c r="D13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E13" t="s">
         <v>41</v>
@@ -1989,7 +1989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>82</v>
       </c>
       <c r="D14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E14" t="s">
         <v>41</v>
@@ -2094,19 +2094,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>57</v>
       </c>
@@ -2132,7 +2132,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -2166,13 +2166,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>72</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -2202,7 +2202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>74</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>75</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>76</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -2290,7 +2290,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>80</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>81</v>
       </c>
@@ -2312,7 +2312,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
Changes Sept 4 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616FD5A7-B7FB-4C0C-9B8C-64ED8781F918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA75D45-3BD5-41B9-B1A5-8CD81464EFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -643,13 +643,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -657,7 +657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -673,12 +673,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -686,7 +686,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -702,17 +702,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -725,17 +725,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -749,15 +749,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -849,7 +849,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -857,7 +857,7 @@
         <v>40</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D2" t="s">
         <v>85</v>
@@ -941,10 +941,10 @@
         <v>56</v>
       </c>
       <c r="AE2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -952,7 +952,7 @@
         <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
         <v>85</v>
@@ -1036,10 +1036,10 @@
         <v>56</v>
       </c>
       <c r="AE3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -1047,7 +1047,7 @@
         <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
         <v>85</v>
@@ -1131,10 +1131,10 @@
         <v>56</v>
       </c>
       <c r="AE4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>40</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
         <v>85</v>
@@ -1226,10 +1226,10 @@
         <v>56</v>
       </c>
       <c r="AE5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
         <v>85</v>
@@ -1321,10 +1321,10 @@
         <v>56</v>
       </c>
       <c r="AE6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>40</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" t="s">
         <v>85</v>
@@ -1416,10 +1416,10 @@
         <v>56</v>
       </c>
       <c r="AE7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>40</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" t="s">
         <v>85</v>
@@ -1511,10 +1511,10 @@
         <v>56</v>
       </c>
       <c r="AE8">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>40</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" t="s">
         <v>85</v>
@@ -1606,10 +1606,10 @@
         <v>56</v>
       </c>
       <c r="AE9">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>40</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
         <v>85</v>
@@ -1701,10 +1701,10 @@
         <v>56</v>
       </c>
       <c r="AE10">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>40</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D11" t="s">
         <v>85</v>
@@ -1796,10 +1796,10 @@
         <v>56</v>
       </c>
       <c r="AE11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -2094,19 +2094,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>57</v>
       </c>
@@ -2132,7 +2132,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -2166,13 +2166,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -2180,117 +2180,117 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>72</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>72</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>69</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>70</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>71</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>71</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>73</v>
-      </c>
-      <c r="B5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>74</v>
       </c>
       <c r="B6" t="s">
         <v>83</v>
       </c>
       <c r="C6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
         <v>83</v>
       </c>
       <c r="C7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
         <v>83</v>
       </c>
       <c r="C8">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
         <v>83</v>
       </c>
       <c r="C9">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" t="s">
         <v>83</v>
       </c>
       <c r="C10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>80</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>81</v>
       </c>
@@ -2312,7 +2312,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
Compliance+Legal +Outlook change  4/8/2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304A8E7C-8A41-4E26-9EF4-8B805DFEEF07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEEE4AD-8D87-4A26-A356-CCDFD7F3D2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="AddOpportunity" sheetId="12" r:id="rId5"/>
     <sheet name="AddContact" sheetId="14" r:id="rId6"/>
     <sheet name="Engagement" sheetId="15" r:id="rId7"/>
+    <sheet name="Notes" sheetId="16" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="93">
   <si>
     <t>James Craven</t>
   </si>
@@ -303,6 +304,24 @@
   </si>
   <si>
     <t>Brian Miller</t>
+  </si>
+  <si>
+    <t>Compliance User</t>
+  </si>
+  <si>
+    <t>Lorriane Johnson</t>
+  </si>
+  <si>
+    <t>Legal User</t>
+  </si>
+  <si>
+    <t>Christine Sha</t>
+  </si>
+  <si>
+    <t>Legal Hold test Notes</t>
+  </si>
+  <si>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
@@ -1063,10 +1082,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1083,6 +1103,22 @@
       </c>
       <c r="B2" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -2723,4 +2759,27 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compliance&Legal Opp users FVA&FR
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEEE4AD-8D87-4A26-A356-CCDFD7F3D2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEFB259-D45E-494A-AD05-8A6DE5AFEBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
user updated 16 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEFB259-D45E-494A-AD05-8A6DE5AFEBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{871296EA-C918-4C9B-8FE0-9D00F7C5A810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -303,9 +303,6 @@
     <t>Engagements</t>
   </si>
   <si>
-    <t>Brian Miller</t>
-  </si>
-  <si>
     <t>Compliance User</t>
   </si>
   <si>
@@ -322,6 +319,9 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>Jennie Stewart</t>
   </si>
 </sst>
 </file>
@@ -1053,13 +1053,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1083,13 +1083,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1097,28 +1097,28 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" t="s">
         <v>88</v>
-      </c>
-      <c r="B3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1129,17 +1129,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1152,22 +1152,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>85</v>
       </c>
@@ -1181,15 +1181,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>39</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -2526,19 +2526,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -2598,13 +2598,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -2612,7 +2612,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>68</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>72</v>
       </c>
@@ -2667,7 +2667,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>74</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>79</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>80</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>81</v>
       </c>
@@ -2764,19 +2764,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Summer release June 17 2025 changes_!
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{871296EA-C918-4C9B-8FE0-9D00F7C5A810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80635F8-DB1A-4050-9DC4-833EB182F8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -1053,13 +1053,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1083,13 +1083,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>92</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -1113,7 +1113,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -1129,17 +1129,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1152,22 +1152,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>85</v>
       </c>
@@ -1180,16 +1180,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
-  <dimension ref="A1:AE14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AD14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -1372,11 +1372,8 @@
       <c r="AD2" t="s">
         <v>55</v>
       </c>
-      <c r="AE2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -1467,11 +1464,8 @@
       <c r="AD3" t="s">
         <v>55</v>
       </c>
-      <c r="AE3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -1562,11 +1556,8 @@
       <c r="AD4" t="s">
         <v>55</v>
       </c>
-      <c r="AE4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1657,11 +1648,8 @@
       <c r="AD5" t="s">
         <v>55</v>
       </c>
-      <c r="AE5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1752,11 +1740,8 @@
       <c r="AD6" t="s">
         <v>55</v>
       </c>
-      <c r="AE6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1847,11 +1832,8 @@
       <c r="AD7" t="s">
         <v>55</v>
       </c>
-      <c r="AE7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>39</v>
       </c>
@@ -1942,11 +1924,8 @@
       <c r="AD8" t="s">
         <v>55</v>
       </c>
-      <c r="AE8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -2037,11 +2016,8 @@
       <c r="AD9" t="s">
         <v>55</v>
       </c>
-      <c r="AE9">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -2132,11 +2108,8 @@
       <c r="AD10" t="s">
         <v>55</v>
       </c>
-      <c r="AE10">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -2227,11 +2200,8 @@
       <c r="AD11" t="s">
         <v>55</v>
       </c>
-      <c r="AE11">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -2322,11 +2292,8 @@
       <c r="AD12" t="s">
         <v>55</v>
       </c>
-      <c r="AE12">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -2417,11 +2384,8 @@
       <c r="AD13" t="s">
         <v>55</v>
       </c>
-      <c r="AE13">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -2511,9 +2475,6 @@
       </c>
       <c r="AD14" t="s">
         <v>55</v>
-      </c>
-      <c r="AE14">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2526,19 +2487,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -2564,7 +2525,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -2598,13 +2559,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -2612,7 +2573,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -2623,7 +2584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -2634,7 +2595,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>68</v>
       </c>
@@ -2645,7 +2606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -2656,7 +2617,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>72</v>
       </c>
@@ -2667,7 +2628,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -2678,7 +2639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>74</v>
       </c>
@@ -2689,7 +2650,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -2700,7 +2661,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -2711,7 +2672,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -2722,7 +2683,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>79</v>
       </c>
@@ -2733,7 +2694,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>80</v>
       </c>
@@ -2744,7 +2705,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>81</v>
       </c>
@@ -2764,17 +2725,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>90</v>
       </c>

</xml_diff>

<commit_message>
Summer release change june 18 _2
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80635F8-DB1A-4050-9DC4-833EB182F8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC655F3E-6F2C-46E4-9F74-177A69780700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -252,9 +252,6 @@
     <t>Lender Education</t>
   </si>
   <si>
-    <t>Capital Markets</t>
-  </si>
-  <si>
     <t>Buyside</t>
   </si>
   <si>
@@ -322,6 +319,9 @@
   </si>
   <si>
     <t>Jennie Stewart</t>
+  </si>
+  <si>
+    <t>Capital Solutions</t>
   </si>
 </sst>
 </file>
@@ -1099,7 +1099,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -1107,18 +1107,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1169,7 +1169,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1200,7 +1200,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1289,10 +1289,10 @@
         <v>39</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
@@ -1381,10 +1381,10 @@
         <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E3" t="s">
         <v>40</v>
@@ -1476,7 +1476,7 @@
         <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E4" t="s">
         <v>40</v>
@@ -1565,10 +1565,10 @@
         <v>39</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E5" t="s">
         <v>40</v>
@@ -1657,10 +1657,10 @@
         <v>39</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E6" t="s">
         <v>40</v>
@@ -1749,10 +1749,10 @@
         <v>39</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
         <v>40</v>
@@ -1841,10 +1841,10 @@
         <v>39</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E8" t="s">
         <v>40</v>
@@ -1933,10 +1933,10 @@
         <v>39</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E9" t="s">
         <v>40</v>
@@ -2025,10 +2025,10 @@
         <v>39</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E10" t="s">
         <v>40</v>
@@ -2117,10 +2117,10 @@
         <v>39</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
         <v>40</v>
@@ -2209,10 +2209,10 @@
         <v>39</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E12" t="s">
         <v>40</v>
@@ -2301,10 +2301,10 @@
         <v>39</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
         <v>40</v>
@@ -2393,10 +2393,10 @@
         <v>39</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E14" t="s">
         <v>40</v>
@@ -2575,10 +2575,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2">
         <v>10</v>
@@ -2586,10 +2586,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -2600,7 +2600,7 @@
         <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2608,10 +2608,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -2619,10 +2619,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -2630,10 +2630,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -2641,10 +2641,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C8">
         <v>6</v>
@@ -2652,10 +2652,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C9">
         <v>7</v>
@@ -2663,10 +2663,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C10">
         <v>8</v>
@@ -2674,10 +2674,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C11">
         <v>9</v>
@@ -2685,10 +2685,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C12">
         <v>11</v>
@@ -2696,10 +2696,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C13">
         <v>12</v>
@@ -2707,10 +2707,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="C14">
         <v>13</v>
@@ -2732,12 +2732,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Summer release June 2125 changes Final
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC655F3E-6F2C-46E4-9F74-177A69780700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6952F996-E6C5-4BF1-9F15-1960AAC2D565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -279,15 +279,6 @@
     <t>Activism Advisory</t>
   </si>
   <si>
-    <t>Strategy</t>
-  </si>
-  <si>
-    <t>Post Merger Integration</t>
-  </si>
-  <si>
-    <t>Valuation Advisory</t>
-  </si>
-  <si>
     <t>Advisory (CF)</t>
   </si>
   <si>
@@ -319,6 +310,15 @@
   </si>
   <si>
     <t>Jennie Stewart</t>
+  </si>
+  <si>
+    <t>Debt Financing</t>
+  </si>
+  <si>
+    <t>Directs</t>
+  </si>
+  <si>
+    <t>Primary Capital Advisory</t>
   </si>
   <si>
     <t>Capital Solutions</t>
@@ -716,20 +716,14 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyFont="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{18F405CE-23A4-4C4C-B371-AE456DF50166}"/>
@@ -1099,7 +1093,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -1107,18 +1101,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1169,7 +1163,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1200,7 +1194,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1292,7 +1286,7 @@
         <v>77</v>
       </c>
       <c r="D2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
@@ -1384,7 +1378,7 @@
         <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E3" t="s">
         <v>40</v>
@@ -1476,7 +1470,7 @@
         <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
         <v>40</v>
@@ -1568,7 +1562,7 @@
         <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
         <v>40</v>
@@ -1656,11 +1650,11 @@
       <c r="B6" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E6" t="s">
         <v>40</v>
@@ -1748,11 +1742,11 @@
       <c r="B7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E7" t="s">
         <v>40</v>
@@ -1840,11 +1834,11 @@
       <c r="B8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>73</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
         <v>40</v>
@@ -1932,11 +1926,11 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>74</v>
       </c>
       <c r="D9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
         <v>40</v>
@@ -2024,11 +2018,11 @@
       <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
         <v>40</v>
@@ -2116,11 +2110,11 @@
       <c r="B11" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>76</v>
       </c>
       <c r="D11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E11" t="s">
         <v>40</v>
@@ -2208,11 +2202,11 @@
       <c r="B12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>78</v>
+      <c r="C12" t="s">
+        <v>89</v>
       </c>
       <c r="D12" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E12" t="s">
         <v>40</v>
@@ -2300,11 +2294,11 @@
       <c r="B13" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>79</v>
+      <c r="C13" t="s">
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E13" t="s">
         <v>40</v>
@@ -2392,11 +2386,11 @@
       <c r="B14" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" t="s">
         <v>80</v>
-      </c>
-      <c r="D14" t="s">
-        <v>83</v>
       </c>
       <c r="E14" t="s">
         <v>40</v>
@@ -2581,7 +2575,7 @@
         <v>77</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2622,7 +2616,7 @@
         <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -2633,7 +2627,7 @@
         <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -2644,7 +2638,7 @@
         <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C8">
         <v>6</v>
@@ -2655,7 +2649,7 @@
         <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C9">
         <v>7</v>
@@ -2666,7 +2660,7 @@
         <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C10">
         <v>8</v>
@@ -2677,43 +2671,43 @@
         <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C11">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>81</v>
+      <c r="A12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" t="s">
+        <v>92</v>
       </c>
       <c r="C12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C13">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14">
         <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2732,12 +2726,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Company IP test cases july 8 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6952F996-E6C5-4BF1-9F15-1960AAC2D565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7471374-94CD-4939-B800-CF8004C94A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Gift Logs+ TMTI0120008 TMTI0120042 TMTI0120019 TMTI0120011 TMTI0120025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017E15C5-FD70-46CB-BCCF-FDC6B5D2F955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41ABA873-F224-472B-AE40-C8F907938BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="AddOpportunity" sheetId="12" r:id="rId5"/>
     <sheet name="AddContact" sheetId="14" r:id="rId6"/>
     <sheet name="Engagement" sheetId="15" r:id="rId7"/>
-    <sheet name="Notes" sheetId="16" r:id="rId8"/>
+    <sheet name="ProductType" sheetId="17" r:id="rId8"/>
+    <sheet name="Notes" sheetId="16" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="104">
   <si>
     <t>James Craven</t>
   </si>
@@ -267,9 +268,6 @@
     <t>Real Estate Brokerage</t>
   </si>
   <si>
-    <t>Special Committee Advisory</t>
-  </si>
-  <si>
     <t>Strategic Alternatives Study</t>
   </si>
   <si>
@@ -322,13 +320,49 @@
   </si>
   <si>
     <t>Capital Solutions</t>
+  </si>
+  <si>
+    <t>Equity Placements</t>
+  </si>
+  <si>
+    <t>GP Stake Sale</t>
+  </si>
+  <si>
+    <t>LP-Led Secondaries</t>
+  </si>
+  <si>
+    <t>Liability Management</t>
+  </si>
+  <si>
+    <t>Advisory</t>
+  </si>
+  <si>
+    <t>ProductType</t>
+  </si>
+  <si>
+    <t>ERPProductTypeCode</t>
+  </si>
+  <si>
+    <t>ADV</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>Ajay Nair</t>
+  </si>
+  <si>
+    <t>System Admin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -463,6 +497,12 @@
       <sz val="11"/>
       <color indexed="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -710,13 +750,14 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyFont="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{18F405CE-23A4-4C4C-B371-AE456DF50166}"/>
@@ -1069,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -1086,7 +1127,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -1094,18 +1135,26 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1156,7 +1205,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1167,7 +1216,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
-  <dimension ref="A1:AD14"/>
+  <dimension ref="A1:AD17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
@@ -1187,7 +1236,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1276,10 +1325,10 @@
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
@@ -1371,7 +1420,7 @@
         <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
         <v>40</v>
@@ -1463,7 +1512,7 @@
         <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
         <v>40</v>
@@ -1555,7 +1604,7 @@
         <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E5" t="s">
         <v>40</v>
@@ -1647,7 +1696,7 @@
         <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E6" t="s">
         <v>40</v>
@@ -1739,7 +1788,7 @@
         <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E7" t="s">
         <v>40</v>
@@ -1831,7 +1880,7 @@
         <v>73</v>
       </c>
       <c r="D8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E8" t="s">
         <v>40</v>
@@ -1920,10 +1969,10 @@
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="D9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E9" t="s">
         <v>40</v>
@@ -2012,10 +2061,10 @@
         <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E10" t="s">
         <v>40</v>
@@ -2104,10 +2153,10 @@
         <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E11" t="s">
         <v>40</v>
@@ -2196,10 +2245,10 @@
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E12" t="s">
         <v>40</v>
@@ -2288,10 +2337,10 @@
         <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E13" t="s">
         <v>40</v>
@@ -2380,10 +2429,10 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E14" t="s">
         <v>40</v>
@@ -2461,6 +2510,282 @@
         <v>0</v>
       </c>
       <c r="AD14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" t="s">
+        <v>41</v>
+      </c>
+      <c r="G15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" t="s">
+        <v>42</v>
+      </c>
+      <c r="I15" t="s">
+        <v>41</v>
+      </c>
+      <c r="J15" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" t="s">
+        <v>43</v>
+      </c>
+      <c r="L15" t="s">
+        <v>44</v>
+      </c>
+      <c r="M15" t="s">
+        <v>45</v>
+      </c>
+      <c r="N15" t="s">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="R15" t="s">
+        <v>47</v>
+      </c>
+      <c r="S15" t="s">
+        <v>47</v>
+      </c>
+      <c r="T15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U15" t="s">
+        <v>49</v>
+      </c>
+      <c r="V15" t="s">
+        <v>50</v>
+      </c>
+      <c r="W15" t="s">
+        <v>51</v>
+      </c>
+      <c r="X15" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" t="s">
+        <v>42</v>
+      </c>
+      <c r="I16" t="s">
+        <v>41</v>
+      </c>
+      <c r="J16" t="s">
+        <v>41</v>
+      </c>
+      <c r="K16" t="s">
+        <v>43</v>
+      </c>
+      <c r="L16" t="s">
+        <v>44</v>
+      </c>
+      <c r="M16" t="s">
+        <v>45</v>
+      </c>
+      <c r="N16" t="s">
+        <v>0</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="R16" t="s">
+        <v>47</v>
+      </c>
+      <c r="S16" t="s">
+        <v>47</v>
+      </c>
+      <c r="T16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U16" t="s">
+        <v>49</v>
+      </c>
+      <c r="V16" t="s">
+        <v>50</v>
+      </c>
+      <c r="W16" t="s">
+        <v>51</v>
+      </c>
+      <c r="X16" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" t="s">
+        <v>41</v>
+      </c>
+      <c r="G17" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17" t="s">
+        <v>41</v>
+      </c>
+      <c r="J17" t="s">
+        <v>41</v>
+      </c>
+      <c r="K17" t="s">
+        <v>43</v>
+      </c>
+      <c r="L17" t="s">
+        <v>44</v>
+      </c>
+      <c r="M17" t="s">
+        <v>45</v>
+      </c>
+      <c r="N17" t="s">
+        <v>0</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="R17" t="s">
+        <v>47</v>
+      </c>
+      <c r="S17" t="s">
+        <v>47</v>
+      </c>
+      <c r="T17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U17" t="s">
+        <v>49</v>
+      </c>
+      <c r="V17" t="s">
+        <v>50</v>
+      </c>
+      <c r="W17" t="s">
+        <v>51</v>
+      </c>
+      <c r="X17" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2545,7 +2870,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -2562,10 +2887,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2">
         <v>13</v>
@@ -2587,7 +2912,7 @@
         <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2609,7 +2934,7 @@
         <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -2620,7 +2945,7 @@
         <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -2631,7 +2956,7 @@
         <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C8">
         <v>6</v>
@@ -2639,10 +2964,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="C9">
         <v>7</v>
@@ -2650,10 +2975,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C10">
         <v>8</v>
@@ -2661,10 +2986,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C11">
         <v>9</v>
@@ -2672,10 +2997,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C12">
         <v>10</v>
@@ -2683,10 +3008,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C13">
         <v>11</v>
@@ -2694,13 +3019,46 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" t="s">
         <v>91</v>
-      </c>
-      <c r="B14" t="s">
-        <v>92</v>
       </c>
       <c r="C14">
         <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2710,6 +3068,156 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCF8D60A-1002-4D00-B235-C15EB6546928}">
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2719,12 +3227,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CSOpp jobtypes minor changes aept 2 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41ABA873-F224-472B-AE40-C8F907938BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49B353A-74CB-42B3-AAC8-BDE2D3EBB6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -1968,7 +1968,7 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>92</v>
       </c>
       <c r="D9" t="s">

</xml_diff>

<commit_message>
Sept 3 2025 minor chabges FS use FS OPp/Eng
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49B353A-74CB-42B3-AAC8-BDE2D3EBB6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D1C60C-5E0B-4CDC-8B2F-ABFD2C74999C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -750,7 +750,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyFont="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -758,6 +758,7 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{18F405CE-23A4-4C4C-B371-AE456DF50166}"/>
@@ -1968,7 +1969,7 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="5" t="s">
         <v>92</v>
       </c>
       <c r="D9" t="s">

</xml_diff>

<commit_message>
Sept 10 2025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
+++ b/TestData/LV_T1426_OpportunityToEngagementConversionMappingForCF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D1C60C-5E0B-4CDC-8B2F-ABFD2C74999C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE11E111-F8BE-4CA7-9905-900913ED4A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -750,7 +750,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyFont="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -758,7 +758,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{18F405CE-23A4-4C4C-B371-AE456DF50166}"/>
@@ -1326,7 +1325,7 @@
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="D2" t="s">
         <v>79</v>
@@ -1418,7 +1417,7 @@
         <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
         <v>79</v>
@@ -1510,7 +1509,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
         <v>79</v>
@@ -1602,7 +1601,7 @@
         <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
         <v>79</v>
@@ -1694,7 +1693,7 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
         <v>79</v>
@@ -1786,7 +1785,7 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
         <v>79</v>
@@ -1878,7 +1877,7 @@
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D8" t="s">
         <v>79</v>
@@ -1969,8 +1968,8 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>92</v>
+      <c r="C9" t="s">
+        <v>70</v>
       </c>
       <c r="D9" t="s">
         <v>79</v>
@@ -2062,7 +2061,7 @@
         <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D10" t="s">
         <v>79</v>
@@ -2154,7 +2153,7 @@
         <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
         <v>79</v>
@@ -2246,7 +2245,7 @@
         <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
         <v>79</v>
@@ -2338,7 +2337,7 @@
         <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
         <v>79</v>
@@ -2430,7 +2429,7 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
         <v>79</v>
@@ -2522,7 +2521,7 @@
         <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D15" t="s">
         <v>79</v>
@@ -2614,7 +2613,7 @@
         <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="D16" t="s">
         <v>79</v>
@@ -2706,7 +2705,7 @@
         <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="D17" t="s">
         <v>79</v>
@@ -2888,178 +2887,178 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C2">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
         <v>91</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="C7">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C8">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="C9">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C11">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C12">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C14">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
         <v>91</v>
       </c>
       <c r="C15">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C16">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C17">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3087,18 +3086,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3111,26 +3110,26 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3143,50 +3142,50 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3199,18 +3198,18 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>